<commit_message>
arquivos FT e RDO
arquivos FT e RDO
</commit_message>
<xml_diff>
--- a/saida_relatorios/Eletrogóes_S_A/Supervisório_UHE_Rondon/RDO_2026-05.xlsx
+++ b/saida_relatorios/Eletrogóes_S_A/Supervisório_UHE_Rondon/RDO_2026-05.xlsx
@@ -4101,7 +4101,7 @@
       </c>
       <c r="K4" s="70" t="inlineStr">
         <is>
-          <t>1 de 13</t>
+          <t>1 de 14</t>
         </is>
       </c>
     </row>
@@ -16172,7 +16172,7 @@
       </c>
       <c r="K1" s="62" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -16220,7 +16220,7 @@
       </c>
       <c r="K4" s="70" t="inlineStr">
         <is>
-          <t>7 de 13</t>
+          <t>8 de 14</t>
         </is>
       </c>
     </row>
@@ -17382,7 +17382,7 @@
       </c>
       <c r="K1" s="62" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -17430,7 +17430,7 @@
       </c>
       <c r="K4" s="70" t="inlineStr">
         <is>
-          <t>8 de 13</t>
+          <t>9 de 14</t>
         </is>
       </c>
     </row>

</xml_diff>